<commit_message>
chore: limpia temporales gude-*.log del repo, corrige SCA browserslist y sube cambios de staff/customers/content
- SCA: override browserslist ^4.28.7 en pnpm-workspace.yaml (fix CVE-2025-53960 / GHSA-c83g-rgw3-j3cx + GHSA-73wf-gq98-2v4g) -> audit limpio
- .gitignore: nuevo patron **/gude-*.log (temporales de edicion DaVinci/Paint.NET que se colaban en content/)
- Des-trackea 15 gude-*.log que estaban en git (ya no se suben)
- Elimina .nojekyll (no hay GitHub Pages), opencode.json.bak, query (basura accidental)
- Contenido ciszukoantony/ciszubot: rename contorn->contour, thumbnails nuevos, limpieza temporales
- archives/staff y archives/customers: regeneracion de docs (STAFFCON/CUSTOMERSCON)
- pnpm-lock.yaml actualizado (override browserslist)
</commit_message>
<xml_diff>
--- a/archives/customers/docs/CUSTOMERS_GLOBAL.xlsx
+++ b/archives/customers/docs/CUSTOMERS_GLOBAL.xlsx
@@ -89,7 +89,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H4"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
@@ -227,7 +227,49 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr" s="2">
+        <is>
+          <t>CL-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="2">
+        <is>
+          <t>TESTEO</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="2">
+        <is>
+          <t>TESTEA</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="2">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="2">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="2">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="2">
+        <is>
+          <t>test</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="2">
+        <is>
+          <t>inactivo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H3"/>
+  <autoFilter ref="A1:H4"/>
 </worksheet>
 </file>
</xml_diff>